<commit_message>
docs: restore result and notes columns (H/I/J/K) from original test spec
</commit_message>
<xml_diff>
--- a/docs/テスト仕様書/テスト仕様書.xlsx
+++ b/docs/テスト仕様書/テスト仕様書.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\テスト\godufo-game\docs\テスト仕様書\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8D515B-0084-4F03-8E85-AD349EF8A5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1A7608-78A0-49F7-AB3C-504858FF6CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t>システム名</t>
   </si>
@@ -96,6 +96,9 @@
     <t>タイトル画面が消え、isStartedがtrueとなり、Wave 1の敵が生成される</t>
   </si>
   <si>
+    <t>OK</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -150,6 +153,15 @@
     <t>specialEnergyが100の時、全敵にダメージを与えエネルギーが0になる</t>
   </si>
   <si>
+    <t>NG</t>
+  </si>
+  <si>
+    <t>スマホでの使用不可</t>
+  </si>
+  <si>
+    <t>スマホでも必殺技ボタンで使用可能</t>
+  </si>
+  <si>
     <t>異常系</t>
   </si>
   <si>
@@ -355,12 +367,6 @@
   </si>
   <si>
     <t>備考</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>NG</t>
   </si>
   <si>
     <t>その他</t>
@@ -420,7 +426,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD3D3D3" tint="0"/>
+        <fgColor rgb="FFD3D3D3"/>
       </patternFill>
     </fill>
   </fills>
@@ -877,10 +883,10 @@
         <v>24</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -891,19 +897,19 @@
         <v>18</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>24</v>
@@ -912,10 +918,10 @@
         <v>24</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -926,19 +932,19 @@
         <v>18</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>24</v>
@@ -947,10 +953,10 @@
         <v>24</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
@@ -961,19 +967,19 @@
         <v>18</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>24</v>
@@ -982,10 +988,10 @@
         <v>24</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -996,31 +1002,31 @@
         <v>18</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13">
@@ -1028,34 +1034,34 @@
         <v>6</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -1066,19 +1072,19 @@
         <v>18</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>24</v>
@@ -1087,10 +1093,10 @@
         <v>24</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15">
@@ -1101,19 +1107,19 @@
         <v>18</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>24</v>
@@ -1122,10 +1128,10 @@
         <v>24</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -1136,19 +1142,19 @@
         <v>18</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>24</v>
@@ -1157,10 +1163,10 @@
         <v>24</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -1171,19 +1177,19 @@
         <v>18</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>24</v>
@@ -1192,10 +1198,10 @@
         <v>24</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -1206,19 +1212,19 @@
         <v>18</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>24</v>
@@ -1227,10 +1233,10 @@
         <v>24</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -1241,19 +1247,19 @@
         <v>18</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>24</v>
@@ -1262,10 +1268,10 @@
         <v>24</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -1276,19 +1282,19 @@
         <v>18</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>24</v>
@@ -1297,10 +1303,10 @@
         <v>24</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21">
@@ -1311,19 +1317,19 @@
         <v>18</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H21" s="5" t="s">
         <v>24</v>
@@ -1332,10 +1338,10 @@
         <v>24</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22">
@@ -1346,19 +1352,19 @@
         <v>18</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>24</v>
@@ -1367,10 +1373,10 @@
         <v>24</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
@@ -1381,19 +1387,19 @@
         <v>18</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>24</v>
@@ -1402,10 +1408,10 @@
         <v>24</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24">
@@ -1416,19 +1422,19 @@
         <v>18</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>24</v>
@@ -1437,10 +1443,10 @@
         <v>24</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -1451,19 +1457,19 @@
         <v>18</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>24</v>
@@ -1472,10 +1478,10 @@
         <v>24</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26">
@@ -1486,19 +1492,19 @@
         <v>18</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>24</v>
@@ -1507,10 +1513,10 @@
         <v>24</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27">
@@ -1521,19 +1527,19 @@
         <v>18</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>24</v>
@@ -1542,27 +1548,34 @@
         <v>24</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
-  <dataValidations count="3">
-    <dataValidation type="list" sqref="B8:B27" showErrorMessage="1" error="正常系/異常系/その他 から選択してください" errorTitle="入力エラー">
-      <formula1>マスタ!$A$2:$A$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="H8:H27" showErrorMessage="1" error="OK/NG/- から選択してください" errorTitle="入力エラー">
-      <formula1>マスタ!$B$2:$B$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="I8:I27" showErrorMessage="1" error="OK/NG/- から選択してください" errorTitle="入力エラー">
-      <formula1>マスタ!$B$2:$B$4</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" showErrorMessage="1" errorTitle="入力エラー" error="正常系/異常系/その他 から選択してください" xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>マスタ!$A$2:$A$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>B8:B27</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" showErrorMessage="1" errorTitle="入力エラー" error="OK/NG/- から選択してください" xr:uid="{00000000-0002-0000-0000-000001000000}">
+          <x14:formula1>
+            <xm:f>マスタ!$B$2:$B$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>H8:I27</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -1583,19 +1596,19 @@
         <v>7</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1623,23 +1636,23 @@
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>111</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>112</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>